<commit_message>
[Lab2] Modified task approach
</commit_message>
<xml_diff>
--- a/Lab2/Lab2 diagrams.xlsx
+++ b/Lab2/Lab2 diagrams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Універ\3 курс\ПО\PC Labs\Lab2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E48EAE-4EDA-4568-B0C3-C32E93176136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7CED80-6789-4BE0-8784-FA93C6FF1169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,12 +60,6 @@
     <t>10^8</t>
   </si>
   <si>
-    <t>5 * 10^8</t>
-  </si>
-  <si>
-    <t>10^9</t>
-  </si>
-  <si>
     <t>Mutex vs atomic</t>
   </si>
   <si>
@@ -73,6 +67,12 @@
   </si>
   <si>
     <t>Atomic</t>
+  </si>
+  <si>
+    <t>10^4</t>
+  </si>
+  <si>
+    <t>5 * 10^6</t>
   </si>
 </sst>
 </file>
@@ -323,25 +323,25 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>10^4</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10^5</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>10^6</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>5 * 10^6</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>10^7</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>5 * 10^7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>10^8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5 * 10^8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10^9</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -353,25 +353,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>2.598E-3</c:v>
+                  <c:v>3.2550000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5720000000000001E-3</c:v>
+                  <c:v>3.79E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.8245999999999998E-2</c:v>
+                  <c:v>3.5145999999999997E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.1901000000000003E-2</c:v>
+                  <c:v>0.122448</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.107372</c:v>
+                  <c:v>0.20022400000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.50119499999999995</c:v>
+                  <c:v>1.5327869999999999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0147710000000001</c:v>
+                  <c:v>3.1831320000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -804,25 +804,25 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>10^4</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10^5</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>10^6</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>5 * 10^6</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>10^7</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>5 * 10^7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>10^8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5 * 10^8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10^9</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -834,25 +834,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>3.6699999999999998E-4</c:v>
+                  <c:v>3.6000000000000001E-5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.7520000000000001E-3</c:v>
+                  <c:v>3.5799999999999997E-4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.5284999999999997E-2</c:v>
+                  <c:v>3.6930000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.23419200000000001</c:v>
+                  <c:v>1.9140000000000001E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.355682</c:v>
+                  <c:v>3.8024000000000002E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.803347</c:v>
+                  <c:v>0.210368</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.6052179999999998</c:v>
+                  <c:v>0.38550800000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1285,25 +1285,25 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>10^4</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10^5</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>10^6</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>5 * 10^6</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>10^7</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>5 * 10^7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>10^8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5 * 10^8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10^9</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1315,25 +1315,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>4.6540000000000002E-3</c:v>
+                  <c:v>9.1489999999999991E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.5550000000000001E-3</c:v>
+                  <c:v>8.1460000000000005E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.9917000000000001E-2</c:v>
+                  <c:v>2.3747999999999998E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.8710999999999999E-2</c:v>
+                  <c:v>8.8794999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.112399</c:v>
+                  <c:v>0.16969999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.53332500000000005</c:v>
+                  <c:v>0.81086800000000003</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.066835</c:v>
+                  <c:v>1.670328</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1766,25 +1766,25 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>10^4</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10^5</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>10^6</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>5 * 10^6</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>10^7</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>5 * 10^7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>10^8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5 * 10^8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10^9</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1796,25 +1796,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>4.6540000000000002E-3</c:v>
+                  <c:v>9.1489999999999991E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.5550000000000001E-3</c:v>
+                  <c:v>8.1460000000000005E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.9917000000000001E-2</c:v>
+                  <c:v>2.3747999999999998E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.8710999999999999E-2</c:v>
+                  <c:v>8.8794999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.112399</c:v>
+                  <c:v>0.16969999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.53332500000000005</c:v>
+                  <c:v>0.81086800000000003</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.066835</c:v>
+                  <c:v>1.670328</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1871,25 +1871,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>2.598E-3</c:v>
+                  <c:v>3.2550000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5720000000000001E-3</c:v>
+                  <c:v>3.79E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.8245999999999998E-2</c:v>
+                  <c:v>3.5145999999999997E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.1901000000000003E-2</c:v>
+                  <c:v>0.122448</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.107372</c:v>
+                  <c:v>0.20022400000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.50119499999999995</c:v>
+                  <c:v>1.5327869999999999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0147710000000001</c:v>
+                  <c:v>3.1831320000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4841,10 +4841,10 @@
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
-        <v>3.6699999999999998E-4</v>
+        <v>3.6000000000000001E-5</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -4853,10 +4853,10 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" s="1">
-        <v>3.7520000000000001E-3</v>
+        <v>3.5799999999999997E-4</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -4865,10 +4865,10 @@
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1">
-        <v>3.5284999999999997E-2</v>
+        <v>3.6930000000000001E-3</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -4877,10 +4877,10 @@
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C8" s="1">
-        <v>0.23419200000000001</v>
+        <v>1.9140000000000001E-2</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -4889,10 +4889,10 @@
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C9" s="1">
-        <v>0.355682</v>
+        <v>3.8024000000000002E-2</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -4901,10 +4901,10 @@
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1">
-        <v>1.803347</v>
+        <v>0.210368</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -4913,10 +4913,10 @@
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1">
-        <v>3.6052179999999998</v>
+        <v>0.38550800000000002</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -4939,58 +4939,58 @@
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C24" s="1">
-        <v>4.6540000000000002E-3</v>
+        <v>9.1489999999999991E-3</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C25" s="1">
-        <v>6.5550000000000001E-3</v>
+        <v>8.1460000000000005E-3</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C26" s="1">
-        <v>1.9917000000000001E-2</v>
+        <v>2.3747999999999998E-2</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C27" s="1">
-        <v>5.8710999999999999E-2</v>
+        <v>8.8794999999999999E-2</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C28" s="1">
-        <v>0.112399</v>
+        <v>0.16969999999999999</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C29" s="1">
-        <v>0.53332500000000005</v>
+        <v>0.81086800000000003</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C30" s="1">
-        <v>1.066835</v>
+        <v>1.670328</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.3">
@@ -5009,63 +5009,63 @@
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B43" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C43" s="1">
-        <v>2.598E-3</v>
+        <v>3.2550000000000001E-3</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B44" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C44" s="1">
-        <v>2.5720000000000001E-3</v>
+        <v>3.79E-3</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B45" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C45" s="1">
-        <v>1.8245999999999998E-2</v>
+        <v>3.5145999999999997E-2</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B46" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C46" s="1">
-        <v>5.1901000000000003E-2</v>
+        <v>0.122448</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B47" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C47" s="1">
-        <v>0.107372</v>
+        <v>0.20022400000000001</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B48" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C48" s="1">
-        <v>0.50119499999999995</v>
+        <v>1.5327869999999999</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B49" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C49" s="1">
-        <v>1.0147710000000001</v>
+        <v>3.1831320000000001</v>
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B60" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="7"/>
@@ -5075,87 +5075,87 @@
         <v>3</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B62" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C62" s="1">
-        <v>4.6540000000000002E-3</v>
+        <v>9.1489999999999991E-3</v>
       </c>
       <c r="D62" s="1">
-        <v>2.598E-3</v>
+        <v>3.2550000000000001E-3</v>
       </c>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B63" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C63" s="1">
-        <v>6.5550000000000001E-3</v>
+        <v>8.1460000000000005E-3</v>
       </c>
       <c r="D63" s="1">
-        <v>2.5720000000000001E-3</v>
+        <v>3.79E-3</v>
       </c>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B64" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C64" s="1">
-        <v>1.9917000000000001E-2</v>
+        <v>2.3747999999999998E-2</v>
       </c>
       <c r="D64" s="1">
-        <v>1.8245999999999998E-2</v>
+        <v>3.5145999999999997E-2</v>
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B65" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C65" s="1">
-        <v>5.8710999999999999E-2</v>
+        <v>8.8794999999999999E-2</v>
       </c>
       <c r="D65" s="1">
-        <v>5.1901000000000003E-2</v>
+        <v>0.122448</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B66" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C66" s="1">
-        <v>0.112399</v>
+        <v>0.16969999999999999</v>
       </c>
       <c r="D66" s="1">
-        <v>0.107372</v>
+        <v>0.20022400000000001</v>
       </c>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B67" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C67" s="1">
-        <v>0.53332500000000005</v>
+        <v>0.81086800000000003</v>
       </c>
       <c r="D67" s="1">
-        <v>0.50119499999999995</v>
+        <v>1.5327869999999999</v>
       </c>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B68" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C68" s="1">
-        <v>1.066835</v>
+        <v>1.670328</v>
       </c>
       <c r="D68" s="1">
-        <v>1.0147710000000001</v>
+        <v>3.1831320000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>